<commit_message>
generated all the reports on 2026-02-22
</commit_message>
<xml_diff>
--- a/report/merged_configurations.xlsx
+++ b/report/merged_configurations.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5353" uniqueCount="1281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5320" uniqueCount="1292">
   <si>
     <t>title</t>
   </si>
@@ -3855,6 +3855,39 @@
   </si>
   <si>
     <t>https://data.vlaanderen.be/doc/concept/StandaardStatus/KandidaatStandaard</t>
+  </si>
+  <si>
+    <t>OSLO SSN SOSA VL</t>
+  </si>
+  <si>
+    <t>https://data.vlaanderen.be/id/concept/StandaardType/Interoperabiliteit</t>
+  </si>
+  <si>
+    <t>SSNSOSA-description.md</t>
+  </si>
+  <si>
+    <t>[{"name":"Datavoorbeelden SSN SOSA VL","resourceReference":"https://github.com/Informatievlaanderen/OSLOthema-SSNSOSA-VL/tree/main/resources"}]</t>
+  </si>
+  <si>
+    <t>Charter SSNSOSAVL</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-SSNSOSA-VL/standaardenregister/charter/Template-Werkgroep-Charter-OSLO.docx</t>
+  </si>
+  <si>
+    <t>[{"name":"Verslag Business Werkgroep - 3 december 2025","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-SSNSOSA-VL/standaardenregister/reports/Verslag%20-%20Business%20werkgroep%20SSN%20SOSA%20VL.pdf"},{"name":"Verslag Thematische Werkgroep 1 - 14 januari 2026","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-SSNSOSA-VL/standaardenregister/reports/Verslag%20Thematische%20werkgroep%201%20-%20SSN%20SOSA%20%202026-02-02.pdf"}]</t>
+  </si>
+  <si>
+    <t>[{"name":"Presentatie Business Werkgroep -  3 december 2025","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-SSNSOSA-VL/standaardenregister/presentations/SSN%20SOSA%20VL%20Business%20Werkgroep.pdf"},{"name":"Presentatie Thematische Werkgroep 1 - 14 januari 2026","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-SSNSOSA-VL/standaardenregister/presentations/Presentatie%20SSN%20SOSA%20VL%20Thematische%20werkgroep%201.pdf"}]</t>
+  </si>
+  <si>
+    <t>https://data.vlaanderen.be/doc/concept/Domein/Omgeving</t>
+  </si>
+  <si>
+    <t>Inspiratiebundel met betrekking tot SSN SOSA VL</t>
+  </si>
+  <si>
+    <t>{"name":"Charter SSNSOSAVL","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-SSNSOSA-VL/standaardenregister/charter/Template-Werkgroep-Charter-OSLO.docx"}</t>
   </si>
 </sst>
 </file>
@@ -4262,7 +4295,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Y258"/>
+  <dimension ref="A1:Y257"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="25" width="44" customWidth="1"/>
@@ -23074,155 +23107,68 @@
     </row>
     <row r="257" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A257" s="3" t="s">
-        <v>37</v>
+        <v>1281</v>
       </c>
       <c r="B257" s="3" t="s">
-        <v>37</v>
+        <v>1282</v>
       </c>
       <c r="C257" s="3" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="D257" s="3" t="s">
-        <v>37</v>
+        <v>767</v>
       </c>
       <c r="E257" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F257" s="3" t="s">
-        <v>37</v>
+        <v>29</v>
+      </c>
+      <c r="F257" s="4">
+        <v>46072</v>
       </c>
       <c r="G257" s="3" t="s">
-        <v>37</v>
+        <v>1283</v>
       </c>
       <c r="H257" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="I257" s="3" t="s">
-        <v>37</v>
+        <v>1284</v>
       </c>
       <c r="J257" s="3" t="s">
-        <v>37</v>
+        <v>1285</v>
       </c>
       <c r="K257" s="3" t="s">
-        <v>37</v>
+        <v>1286</v>
       </c>
       <c r="L257" s="3" t="s">
-        <v>37</v>
+        <v>1287</v>
       </c>
       <c r="M257" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="N257" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="O257" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="P257" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q257" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="R257" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="S257" s="3" t="s">
-        <v>37</v>
-      </c>
+        <v>1288</v>
+      </c>
+      <c r="N257" s="4">
+        <v>45974</v>
+      </c>
+      <c r="O257" s="3"/>
+      <c r="P257" s="3"/>
+      <c r="Q257" s="3"/>
+      <c r="R257" s="3"/>
+      <c r="S257" s="3"/>
       <c r="T257" s="3" t="s">
-        <v>37</v>
+        <v>1289</v>
       </c>
       <c r="U257" s="3" t="s">
         <v>37</v>
       </c>
       <c r="V257" s="3" t="s">
-        <v>37</v>
+        <v>1290</v>
       </c>
       <c r="W257" s="3" t="s">
         <v>37</v>
       </c>
       <c r="X257" s="3" t="s">
-        <v>37</v>
+        <v>1291</v>
       </c>
       <c r="Y257" s="3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="258" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="E258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="G258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="H258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="I258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="J258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="K258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="L258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="M258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="N258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="O258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="P258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="R258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="S258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="T258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="U258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="V258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="W258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="X258" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="Y258" s="3" t="s">
         <v>37</v>
       </c>
     </row>
@@ -23234,7 +23180,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R258"/>
+  <dimension ref="A1:R257"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="18" width="44" customWidth="1"/>
@@ -37578,37 +37524,37 @@
     </row>
     <row r="257" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A257" s="3" t="s">
-        <v>436</v>
-      </c>
-      <c r="B257" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="C257" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="D257" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="E257" s="6" t="b">
-        <v>0</v>
+        <v>1281</v>
+      </c>
+      <c r="B257" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="C257" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="D257" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="E257" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="F257" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G257" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H257" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="I257" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="J257" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="K257" s="6" t="b">
-        <v>0</v>
+      <c r="G257" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H257" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I257" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="J257" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="K257" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="L257" s="6" t="b">
         <v>0</v>
@@ -37625,67 +37571,11 @@
       <c r="P257" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="Q257" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="R257" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="258" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A258" s="3" t="s">
-        <v>436</v>
-      </c>
-      <c r="B258" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="C258" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="D258" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="E258" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F258" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G258" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H258" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="I258" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="J258" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="K258" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="L258" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="M258" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="N258" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="O258" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="P258" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q258" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="R258" s="6" t="b">
-        <v>0</v>
+      <c r="Q257" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="R257" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
generated all the reports on 2026-03-01
</commit_message>
<xml_diff>
--- a/report/merged_configurations.xlsx
+++ b/report/merged_configurations.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5320" uniqueCount="1292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5308" uniqueCount="1291">
   <si>
     <t>title</t>
   </si>
@@ -3852,9 +3852,6 @@
   </si>
   <si>
     <t>Vocabularium Rooilijnplannen</t>
-  </si>
-  <si>
-    <t>https://data.vlaanderen.be/doc/concept/StandaardStatus/KandidaatStandaard</t>
   </si>
   <si>
     <t>OSLO SSN SOSA VL</t>
@@ -15815,7 +15812,7 @@
         <v>27</v>
       </c>
       <c r="D158" s="3" t="s">
-        <v>28</v>
+        <v>63</v>
       </c>
       <c r="E158" s="3" t="s">
         <v>151</v>
@@ -15850,8 +15847,8 @@
       <c r="O158" s="4">
         <v>46030</v>
       </c>
-      <c r="P158" s="3" t="s">
-        <v>121</v>
+      <c r="P158" s="4">
+        <v>46073</v>
       </c>
       <c r="Q158" s="3"/>
       <c r="R158" s="3" t="s">
@@ -15888,7 +15885,7 @@
         <v>27</v>
       </c>
       <c r="D159" s="3" t="s">
-        <v>28</v>
+        <v>63</v>
       </c>
       <c r="E159" s="3" t="s">
         <v>151</v>
@@ -15923,8 +15920,8 @@
       <c r="O159" s="4">
         <v>46030</v>
       </c>
-      <c r="P159" s="3" t="s">
-        <v>121</v>
+      <c r="P159" s="4">
+        <v>46073</v>
       </c>
       <c r="Q159" s="3"/>
       <c r="R159" s="3" t="s">
@@ -15961,7 +15958,7 @@
         <v>27</v>
       </c>
       <c r="D160" s="3" t="s">
-        <v>28</v>
+        <v>63</v>
       </c>
       <c r="E160" s="3" t="s">
         <v>151</v>
@@ -15996,8 +15993,8 @@
       <c r="O160" s="4">
         <v>46030</v>
       </c>
-      <c r="P160" s="3" t="s">
-        <v>121</v>
+      <c r="P160" s="4">
+        <v>46073</v>
       </c>
       <c r="Q160" s="3"/>
       <c r="R160" s="3" t="s">
@@ -19396,7 +19393,7 @@
         <v>27</v>
       </c>
       <c r="D207" s="3" t="s">
-        <v>28</v>
+        <v>63</v>
       </c>
       <c r="E207" s="3" t="s">
         <v>29</v>
@@ -19428,11 +19425,11 @@
       <c r="N207" s="4">
         <v>45974</v>
       </c>
-      <c r="O207" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="P207" s="3" t="s">
-        <v>121</v>
+      <c r="O207" s="4">
+        <v>46030</v>
+      </c>
+      <c r="P207" s="4">
+        <v>46073</v>
       </c>
       <c r="Q207" s="3"/>
       <c r="R207" s="4">
@@ -22810,7 +22807,7 @@
         <v>27</v>
       </c>
       <c r="D253" s="3" t="s">
-        <v>28</v>
+        <v>63</v>
       </c>
       <c r="E253" s="3" t="s">
         <v>29</v>
@@ -22842,11 +22839,11 @@
       <c r="N253" s="4">
         <v>45743</v>
       </c>
-      <c r="O253" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="P253" s="3" t="s">
-        <v>121</v>
+      <c r="O253" s="4">
+        <v>46030</v>
+      </c>
+      <c r="P253" s="4">
+        <v>46065</v>
       </c>
       <c r="Q253" s="4">
         <v>45867</v>
@@ -22854,8 +22851,8 @@
       <c r="R253" s="4">
         <v>45961</v>
       </c>
-      <c r="S253" s="3" t="s">
-        <v>121</v>
+      <c r="S253" s="3">
+        <v>0</v>
       </c>
       <c r="T253" s="3" t="s">
         <v>109</v>
@@ -22887,7 +22884,7 @@
         <v>27</v>
       </c>
       <c r="D254" s="3" t="s">
-        <v>28</v>
+        <v>63</v>
       </c>
       <c r="E254" s="3" t="s">
         <v>29</v>
@@ -22919,11 +22916,11 @@
       <c r="N254" s="4">
         <v>45666</v>
       </c>
-      <c r="O254" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="P254" s="3" t="s">
-        <v>121</v>
+      <c r="O254" s="4">
+        <v>46030</v>
+      </c>
+      <c r="P254" s="4">
+        <v>46065</v>
       </c>
       <c r="Q254" s="4">
         <v>45858</v>
@@ -22964,7 +22961,7 @@
         <v>27</v>
       </c>
       <c r="D255" s="3" t="s">
-        <v>1280</v>
+        <v>63</v>
       </c>
       <c r="E255" s="3" t="s">
         <v>29</v>
@@ -22996,11 +22993,11 @@
       <c r="N255" s="4">
         <v>45666</v>
       </c>
-      <c r="O255" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="P255" s="3" t="s">
-        <v>121</v>
+      <c r="O255" s="4">
+        <v>46030</v>
+      </c>
+      <c r="P255" s="4">
+        <v>46065</v>
       </c>
       <c r="Q255" s="4">
         <v>45858</v>
@@ -23107,10 +23104,10 @@
     </row>
     <row r="257" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A257" s="3" t="s">
+        <v>1280</v>
+      </c>
+      <c r="B257" s="3" t="s">
         <v>1281</v>
-      </c>
-      <c r="B257" s="3" t="s">
-        <v>1282</v>
       </c>
       <c r="C257" s="3" t="s">
         <v>27</v>
@@ -23125,25 +23122,25 @@
         <v>46072</v>
       </c>
       <c r="G257" s="3" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
       <c r="H257" s="3" t="s">
         <v>32</v>
       </c>
       <c r="I257" s="3" t="s">
+        <v>1283</v>
+      </c>
+      <c r="J257" s="3" t="s">
         <v>1284</v>
       </c>
-      <c r="J257" s="3" t="s">
+      <c r="K257" s="3" t="s">
         <v>1285</v>
       </c>
-      <c r="K257" s="3" t="s">
+      <c r="L257" s="3" t="s">
         <v>1286</v>
       </c>
-      <c r="L257" s="3" t="s">
+      <c r="M257" s="3" t="s">
         <v>1287</v>
-      </c>
-      <c r="M257" s="3" t="s">
-        <v>1288</v>
       </c>
       <c r="N257" s="4">
         <v>45974</v>
@@ -23154,19 +23151,19 @@
       <c r="R257" s="3"/>
       <c r="S257" s="3"/>
       <c r="T257" s="3" t="s">
+        <v>1288</v>
+      </c>
+      <c r="U257" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="V257" s="3" t="s">
         <v>1289</v>
       </c>
-      <c r="U257" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="V257" s="3" t="s">
+      <c r="W257" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="X257" s="3" t="s">
         <v>1290</v>
-      </c>
-      <c r="W257" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="X257" s="3" t="s">
-        <v>1291</v>
       </c>
       <c r="Y257" s="3" t="s">
         <v>37</v>
@@ -32015,8 +32012,8 @@
       <c r="L158" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="M158" s="6" t="b">
-        <v>0</v>
+      <c r="M158" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="N158" s="6" t="b">
         <v>0</v>
@@ -32071,8 +32068,8 @@
       <c r="L159" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="M159" s="6" t="b">
-        <v>0</v>
+      <c r="M159" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="N159" s="6" t="b">
         <v>0</v>
@@ -32127,8 +32124,8 @@
       <c r="L160" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="M160" s="6" t="b">
-        <v>0</v>
+      <c r="M160" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="N160" s="6" t="b">
         <v>0</v>
@@ -34756,11 +34753,11 @@
       <c r="K207" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="L207" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="M207" s="6" t="b">
-        <v>0</v>
+      <c r="L207" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M207" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="N207" s="6" t="b">
         <v>0</v>
@@ -37332,11 +37329,11 @@
       <c r="K253" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="L253" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="M253" s="6" t="b">
-        <v>0</v>
+      <c r="L253" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M253" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="N253" s="5" t="b">
         <v>1</v>
@@ -37344,8 +37341,8 @@
       <c r="O253" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="P253" s="6" t="b">
-        <v>0</v>
+      <c r="P253" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="Q253" s="5" t="b">
         <v>1</v>
@@ -37388,11 +37385,11 @@
       <c r="K254" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="L254" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="M254" s="6" t="b">
-        <v>0</v>
+      <c r="L254" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M254" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="N254" s="5" t="b">
         <v>1</v>
@@ -37444,11 +37441,11 @@
       <c r="K255" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="L255" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="M255" s="6" t="b">
-        <v>0</v>
+      <c r="L255" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M255" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="N255" s="5" t="b">
         <v>1</v>
@@ -37524,7 +37521,7 @@
     </row>
     <row r="257" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A257" s="3" t="s">
-        <v>1281</v>
+        <v>1280</v>
       </c>
       <c r="B257" s="5" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
generated all the reports on 2026-04-05
</commit_message>
<xml_diff>
--- a/report/merged_configurations.xlsx
+++ b/report/merged_configurations.xlsx
@@ -134,13 +134,16 @@
     <t>Applicatieprofiel Thermografische Gebouwanalyse</t>
   </si>
   <si>
+    <t>https://data.vlaanderen.be/id/concept/StandaardStatus/ErkendeStandaard</t>
+  </si>
+  <si>
     <t>thermai-description.md</t>
   </si>
   <si>
     <t>[{"name":"Applicatieprofiel Thermografische Gebouwanalyse","resourceReference":"https://data.vlaanderen.be/doc/applicatieprofiel/thermografische-gebouwanalyse"}]</t>
   </si>
   <si>
-    <t>[{"name":"Modelleerrapport","resourceReference":"https://github.com/Informatievlaanderen/OSLOthema-thermAI/blob/main/resources/ModelleerrapportThermAI.pdf"},{"name":"Datavoorbeelden","resourceReference":"https://github.com/Informatievlaanderen/OSLOthema-thermAI/tree/main/resources/Datavoorbeelden"}]</t>
+    <t>[{"name":"Modelleerrapport","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-thermAI/main/resources/ModelleerrapportThermAI.pdf"},{"name":"Datavoorbeelden","resourceReference":"https://github.com/Informatievlaanderen/OSLOthema-thermAI/tree/main/resources/Datavoorbeelden"}]</t>
   </si>
   <si>
     <t>Charter Thermografische Gebouwanalyse</t>
@@ -149,10 +152,10 @@
     <t>https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-thermAI/standaardenregister/charter/Charter_OSLO_thermAI.pdf</t>
   </si>
   <si>
-    <t>[{"name":"Verslag Business werkgroep - 18-02-2025","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-thermAI/standaardenregister/reports/Business%20werkgroep%20CoT%20ThermAI%202025-02-18.pdf"},{"name":"Verslag Thematische Werkgroep 1 - 18-03-2025","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-thermAI/standaardenregister/reports/Thematische%20werkgroep%201%20-%20CoT%20ThermAI%202025-03-18.pdf"},{"name":"Verslag Thematische Werkgroep 2 - 15-04-2025","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-thermAI/standaardenregister/reports/Thematische%20werkgroep%202%20-%20CoT%20ThermAI%202025-04-15.pdf"},{"name":"Verslag Thematische Werkgroep 3 - 15-05-2025","resourceReference":"https://github.com/Informatievlaanderen/OSLOthema-thermAI/blob/standaardenregister/reports/Verslag%20Thematische%20werkgroep%203%20-%20CoT%20ThermAI%202025-04-15.docx.pdf"}]</t>
-  </si>
-  <si>
-    <t>[{"name":"Presentatie Business Werkgroep - 18-02-2025","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-thermAI/standaardenregister/presentations/ThermAI%20Business%20Werkgroep%20(1).pdf"},{"name":"Presentatie Thematische Werkgroep 1 - 18-03-2025","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-thermAI/standaardenregister/presentations/Thematische%20werkgroep%201%20-%20ThermAI.pdf"},{"name":"Presentatie Thematische Werkgroep 2 - 15-04-2025","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-thermAI/standaardenregister/presentations/Thematische%20werkgroep%202%20-%20ThermAI.pdf"},{"name":"Presentatie Thematische Werkgroep 3 - 15-05-2025","resourceReference":"https://github.com/Informatievlaanderen/OSLOthema-thermAI/blob/standaardenregister/presentations/Slides%20-%20Thematische%20werkgroep%203%20-%20ThermAI.pdf"}]</t>
+    <t>[{"name":"Verslag Business werkgroep - 18-02-2025","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-thermAI/standaardenregister/reports/Business%20werkgroep%20CoT%20ThermAI%202025-02-18.pdf"},{"name":"Verslag Thematische Werkgroep 1 - 18-03-2025","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-thermAI/standaardenregister/reports/Thematische%20werkgroep%201%20-%20CoT%20ThermAI%202025-03-18.pdf"},{"name":"Verslag Thematische Werkgroep 2 - 15-04-2025","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-thermAI/standaardenregister/reports/Thematische%20werkgroep%202%20-%20CoT%20ThermAI%202025-04-15.pdf"},{"name":"Verslag Thematische Werkgroep 3 - 15-05-2025","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-thermAI/standaardenregister/reports/Verslag%20Thematische%20werkgroep%203%20-%20CoT%20ThermAI%202025-04-15.docx.pdf"}]</t>
+  </si>
+  <si>
+    <t>[{"name":"Presentatie Business Werkgroep - 18-02-2025","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-thermAI/standaardenregister/presentations/ThermAI%20Business%20Werkgroep%20(1).pdf"},{"name":"Presentatie Thematische Werkgroep 1 - 18-03-2025","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-thermAI/standaardenregister/presentations/Thematische%20werkgroep%201%20-%20ThermAI.pdf"},{"name":"Presentatie Thematische Werkgroep 2 - 15-04-2025","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-thermAI/standaardenregister/presentations/Thematische%20werkgroep%202%20-%20ThermAI.pdf"},{"name":"Presentatie Thematische Werkgroep 3 - 15-05-2025","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-thermAI/standaardenregister/presentations/Slides%20-%20Thematische%20werkgroep%203%20-%20ThermAI.pdf"}]</t>
   </si>
   <si>
     <t>2024-12-1</t>
@@ -201,9 +204,6 @@
   </si>
   <si>
     <t>Applicatieprofiel Energiehuis</t>
-  </si>
-  <si>
-    <t>https://data.vlaanderen.be/id/concept/StandaardStatus/ErkendeStandaard</t>
   </si>
   <si>
     <t>energiehuis-description.md</t>
@@ -4460,40 +4460,42 @@
         <v>27</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>29</v>
       </c>
       <c r="F3" s="4">
-        <v>45799</v>
+        <v>46002</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="O3" s="3"/>
-      <c r="P3" s="3"/>
+      <c r="P3" s="4">
+        <v>46002</v>
+      </c>
       <c r="Q3" s="4">
         <v>45854</v>
       </c>
@@ -4502,7 +4504,7 @@
       </c>
       <c r="S3" s="3"/>
       <c r="T3" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="U3" s="3" t="s">
         <v>37</v>
@@ -4514,7 +4516,7 @@
         <v>37</v>
       </c>
       <c r="X3" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="Y3" s="3" t="s">
         <v>37</v>
@@ -4522,7 +4524,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>26</v>
@@ -4534,31 +4536,31 @@
         <v>28</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F4" s="4">
         <v>45889</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>32</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N4" s="4">
         <v>45428</v>
@@ -4573,19 +4575,19 @@
       </c>
       <c r="S4" s="3"/>
       <c r="T4" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="U4" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="V4" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="W4" s="3" t="s">
         <v>37</v>
       </c>
       <c r="X4" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Y4" s="3" t="s">
         <v>37</v>
@@ -4593,7 +4595,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>26</v>
@@ -4602,7 +4604,7 @@
         <v>27</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>29</v>
@@ -4677,7 +4679,7 @@
         <v>27</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>29</v>
@@ -4752,7 +4754,7 @@
         <v>27</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>80</v>
@@ -4827,7 +4829,7 @@
         <v>27</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>80</v>
@@ -4902,7 +4904,7 @@
         <v>27</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>29</v>
@@ -4973,7 +4975,7 @@
         <v>27</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>29</v>
@@ -5044,7 +5046,7 @@
         <v>27</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>29</v>
@@ -5113,7 +5115,7 @@
         <v>27</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>29</v>
@@ -5182,7 +5184,7 @@
         <v>27</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>115</v>
@@ -5255,7 +5257,7 @@
         <v>27</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>115</v>
@@ -5328,7 +5330,7 @@
         <v>27</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>29</v>
@@ -5403,7 +5405,7 @@
         <v>27</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>29</v>
@@ -5478,7 +5480,7 @@
         <v>27</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>29</v>
@@ -5768,7 +5770,7 @@
         <v>27</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>29</v>
@@ -5843,7 +5845,7 @@
         <v>27</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>29</v>
@@ -5991,7 +5993,7 @@
         <v>27</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>29</v>
@@ -6068,7 +6070,7 @@
         <v>27</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>29</v>
@@ -6145,7 +6147,7 @@
         <v>27</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>29</v>
@@ -6218,7 +6220,7 @@
         <v>27</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>29</v>
@@ -6291,7 +6293,7 @@
         <v>27</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>216</v>
@@ -6364,7 +6366,7 @@
         <v>27</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E29" s="3" t="s">
         <v>216</v>
@@ -7329,7 +7331,7 @@
         <v>27</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E42" s="3" t="s">
         <v>230</v>
@@ -7404,7 +7406,7 @@
         <v>27</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E43" s="3" t="s">
         <v>230</v>
@@ -7625,7 +7627,7 @@
         <v>27</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E46" s="3" t="s">
         <v>230</v>
@@ -7700,7 +7702,7 @@
         <v>27</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E47" s="3" t="s">
         <v>230</v>
@@ -7775,7 +7777,7 @@
         <v>27</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E48" s="3" t="s">
         <v>230</v>
@@ -7850,7 +7852,7 @@
         <v>27</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E49" s="3" t="s">
         <v>230</v>
@@ -7925,7 +7927,7 @@
         <v>27</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E50" s="3" t="s">
         <v>308</v>
@@ -7998,7 +8000,7 @@
         <v>27</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>308</v>
@@ -8363,7 +8365,7 @@
         <v>27</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E56" s="3" t="s">
         <v>349</v>
@@ -8436,7 +8438,7 @@
         <v>27</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E57" s="3" t="s">
         <v>349</v>
@@ -8509,7 +8511,7 @@
         <v>27</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E58" s="3" t="s">
         <v>349</v>
@@ -8582,7 +8584,7 @@
         <v>27</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E59" s="3" t="s">
         <v>349</v>
@@ -8655,7 +8657,7 @@
         <v>27</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E60" s="3" t="s">
         <v>29</v>
@@ -8801,7 +8803,7 @@
         <v>27</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E62" s="3" t="s">
         <v>29</v>
@@ -8947,7 +8949,7 @@
         <v>27</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E64" s="3" t="s">
         <v>29</v>
@@ -9020,7 +9022,7 @@
         <v>27</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E65" s="3" t="s">
         <v>29</v>
@@ -9093,7 +9095,7 @@
         <v>27</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E66" s="3" t="s">
         <v>29</v>
@@ -9239,7 +9241,7 @@
         <v>27</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E68" s="3" t="s">
         <v>414</v>
@@ -9312,7 +9314,7 @@
         <v>27</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E69" s="3" t="s">
         <v>29</v>
@@ -9608,7 +9610,7 @@
         <v>27</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E73" s="3" t="s">
         <v>448</v>
@@ -9681,7 +9683,7 @@
         <v>27</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E74" s="3" t="s">
         <v>448</v>
@@ -9827,7 +9829,7 @@
         <v>27</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E76" s="3" t="s">
         <v>29</v>
@@ -10119,7 +10121,7 @@
         <v>27</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E80" s="3" t="s">
         <v>29</v>
@@ -10192,7 +10194,7 @@
         <v>27</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E81" s="3" t="s">
         <v>29</v>
@@ -10265,7 +10267,7 @@
         <v>27</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E82" s="3" t="s">
         <v>29</v>
@@ -10338,7 +10340,7 @@
         <v>27</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E83" s="3" t="s">
         <v>29</v>
@@ -10411,7 +10413,7 @@
         <v>27</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E84" s="3" t="s">
         <v>29</v>
@@ -10484,7 +10486,7 @@
         <v>27</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E85" s="3" t="s">
         <v>513</v>
@@ -10557,7 +10559,7 @@
         <v>27</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E86" s="3" t="s">
         <v>513</v>
@@ -10776,7 +10778,7 @@
         <v>27</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E89" s="3" t="s">
         <v>540</v>
@@ -10849,7 +10851,7 @@
         <v>27</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E90" s="3" t="s">
         <v>540</v>
@@ -10922,7 +10924,7 @@
         <v>27</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E91" s="3" t="s">
         <v>540</v>
@@ -10995,7 +10997,7 @@
         <v>27</v>
       </c>
       <c r="D92" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E92" s="3" t="s">
         <v>540</v>
@@ -11112,7 +11114,7 @@
       </c>
       <c r="S93" s="3"/>
       <c r="T93" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="U93" s="3" t="s">
         <v>37</v>
@@ -11141,7 +11143,7 @@
         <v>27</v>
       </c>
       <c r="D94" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E94" s="3" t="s">
         <v>29</v>
@@ -11185,7 +11187,7 @@
       </c>
       <c r="S94" s="3"/>
       <c r="T94" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="U94" s="3" t="s">
         <v>37</v>
@@ -11214,7 +11216,7 @@
         <v>27</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E95" s="3" t="s">
         <v>29</v>
@@ -11287,7 +11289,7 @@
         <v>27</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E96" s="3" t="s">
         <v>29</v>
@@ -11360,7 +11362,7 @@
         <v>27</v>
       </c>
       <c r="D97" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E97" s="3" t="s">
         <v>595</v>
@@ -11433,7 +11435,7 @@
         <v>27</v>
       </c>
       <c r="D98" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E98" s="3" t="s">
         <v>595</v>
@@ -11506,7 +11508,7 @@
         <v>27</v>
       </c>
       <c r="D99" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E99" s="3" t="s">
         <v>595</v>
@@ -11579,7 +11581,7 @@
         <v>27</v>
       </c>
       <c r="D100" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E100" s="3" t="s">
         <v>595</v>
@@ -11652,7 +11654,7 @@
         <v>27</v>
       </c>
       <c r="D101" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E101" s="3" t="s">
         <v>616</v>
@@ -11725,7 +11727,7 @@
         <v>625</v>
       </c>
       <c r="D102" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E102" s="3" t="s">
         <v>616</v>
@@ -11798,7 +11800,7 @@
         <v>27</v>
       </c>
       <c r="D103" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E103" s="3" t="s">
         <v>616</v>
@@ -11871,7 +11873,7 @@
         <v>625</v>
       </c>
       <c r="D104" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E104" s="3" t="s">
         <v>616</v>
@@ -11944,7 +11946,7 @@
         <v>625</v>
       </c>
       <c r="D105" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E105" s="3" t="s">
         <v>616</v>
@@ -12017,7 +12019,7 @@
         <v>643</v>
       </c>
       <c r="D106" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E106" s="3" t="s">
         <v>29</v>
@@ -12061,7 +12063,7 @@
       </c>
       <c r="S106" s="3"/>
       <c r="T106" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="U106" s="3" t="s">
         <v>37</v>
@@ -12090,7 +12092,7 @@
         <v>643</v>
       </c>
       <c r="D107" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E107" s="3" t="s">
         <v>29</v>
@@ -12134,7 +12136,7 @@
       </c>
       <c r="S107" s="3"/>
       <c r="T107" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="U107" s="3" t="s">
         <v>37</v>
@@ -12163,7 +12165,7 @@
         <v>27</v>
       </c>
       <c r="D108" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E108" s="3" t="s">
         <v>29</v>
@@ -12207,7 +12209,7 @@
       </c>
       <c r="S108" s="3"/>
       <c r="T108" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="U108" s="3" t="s">
         <v>37</v>
@@ -12236,7 +12238,7 @@
         <v>27</v>
       </c>
       <c r="D109" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E109" s="3" t="s">
         <v>29</v>
@@ -12309,7 +12311,7 @@
         <v>27</v>
       </c>
       <c r="D110" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E110" s="3" t="s">
         <v>29</v>
@@ -12382,7 +12384,7 @@
         <v>27</v>
       </c>
       <c r="D111" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E111" s="3" t="s">
         <v>29</v>
@@ -12455,7 +12457,7 @@
         <v>27</v>
       </c>
       <c r="D112" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E112" s="3" t="s">
         <v>29</v>
@@ -12528,7 +12530,7 @@
         <v>27</v>
       </c>
       <c r="D113" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E113" s="3" t="s">
         <v>29</v>
@@ -12601,7 +12603,7 @@
         <v>27</v>
       </c>
       <c r="D114" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E114" s="3" t="s">
         <v>29</v>
@@ -12674,7 +12676,7 @@
         <v>27</v>
       </c>
       <c r="D115" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E115" s="3" t="s">
         <v>29</v>
@@ -12747,7 +12749,7 @@
         <v>27</v>
       </c>
       <c r="D116" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E116" s="3" t="s">
         <v>29</v>
@@ -12820,7 +12822,7 @@
         <v>27</v>
       </c>
       <c r="D117" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E117" s="3" t="s">
         <v>29</v>
@@ -12893,7 +12895,7 @@
         <v>27</v>
       </c>
       <c r="D118" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E118" s="3" t="s">
         <v>29</v>
@@ -12966,7 +12968,7 @@
         <v>27</v>
       </c>
       <c r="D119" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E119" s="3" t="s">
         <v>29</v>
@@ -13039,7 +13041,7 @@
         <v>27</v>
       </c>
       <c r="D120" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E120" s="3" t="s">
         <v>29</v>
@@ -13112,7 +13114,7 @@
         <v>27</v>
       </c>
       <c r="D121" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E121" s="3" t="s">
         <v>29</v>
@@ -13185,7 +13187,7 @@
         <v>27</v>
       </c>
       <c r="D122" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E122" s="3" t="s">
         <v>29</v>
@@ -13258,7 +13260,7 @@
         <v>27</v>
       </c>
       <c r="D123" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E123" s="3" t="s">
         <v>29</v>
@@ -13331,7 +13333,7 @@
         <v>27</v>
       </c>
       <c r="D124" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E124" s="3" t="s">
         <v>29</v>
@@ -13477,7 +13479,7 @@
         <v>27</v>
       </c>
       <c r="D126" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E126" s="3" t="s">
         <v>414</v>
@@ -13550,7 +13552,7 @@
         <v>27</v>
       </c>
       <c r="D127" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E127" s="3" t="s">
         <v>414</v>
@@ -13623,7 +13625,7 @@
         <v>27</v>
       </c>
       <c r="D128" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E128" s="3" t="s">
         <v>308</v>
@@ -13696,7 +13698,7 @@
         <v>27</v>
       </c>
       <c r="D129" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E129" s="3" t="s">
         <v>308</v>
@@ -13769,7 +13771,7 @@
         <v>27</v>
       </c>
       <c r="D130" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E130" s="3" t="s">
         <v>308</v>
@@ -14205,7 +14207,7 @@
         <v>27</v>
       </c>
       <c r="D136" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E136" s="3" t="s">
         <v>29</v>
@@ -14278,7 +14280,7 @@
         <v>27</v>
       </c>
       <c r="D137" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E137" s="3" t="s">
         <v>29</v>
@@ -14351,7 +14353,7 @@
         <v>27</v>
       </c>
       <c r="D138" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E138" s="3" t="s">
         <v>29</v>
@@ -14424,7 +14426,7 @@
         <v>27</v>
       </c>
       <c r="D139" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E139" s="3" t="s">
         <v>29</v>
@@ -14497,7 +14499,7 @@
         <v>27</v>
       </c>
       <c r="D140" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E140" s="3" t="s">
         <v>29</v>
@@ -14570,7 +14572,7 @@
         <v>27</v>
       </c>
       <c r="D141" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E141" s="3" t="s">
         <v>29</v>
@@ -14643,7 +14645,7 @@
         <v>27</v>
       </c>
       <c r="D142" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E142" s="3" t="s">
         <v>29</v>
@@ -14716,7 +14718,7 @@
         <v>27</v>
       </c>
       <c r="D143" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E143" s="3" t="s">
         <v>29</v>
@@ -14789,7 +14791,7 @@
         <v>27</v>
       </c>
       <c r="D144" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E144" s="3" t="s">
         <v>29</v>
@@ -14862,7 +14864,7 @@
         <v>27</v>
       </c>
       <c r="D145" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E145" s="3" t="s">
         <v>29</v>
@@ -14935,7 +14937,7 @@
         <v>27</v>
       </c>
       <c r="D146" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E146" s="3" t="s">
         <v>29</v>
@@ -15008,7 +15010,7 @@
         <v>27</v>
       </c>
       <c r="D147" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E147" s="3" t="s">
         <v>29</v>
@@ -15081,7 +15083,7 @@
         <v>27</v>
       </c>
       <c r="D148" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E148" s="3" t="s">
         <v>29</v>
@@ -15154,7 +15156,7 @@
         <v>27</v>
       </c>
       <c r="D149" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E149" s="3" t="s">
         <v>29</v>
@@ -15227,7 +15229,7 @@
         <v>27</v>
       </c>
       <c r="D150" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E150" s="3" t="s">
         <v>29</v>
@@ -15300,7 +15302,7 @@
         <v>27</v>
       </c>
       <c r="D151" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E151" s="3" t="s">
         <v>29</v>
@@ -15373,7 +15375,7 @@
         <v>27</v>
       </c>
       <c r="D152" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E152" s="3" t="s">
         <v>29</v>
@@ -15446,7 +15448,7 @@
         <v>27</v>
       </c>
       <c r="D153" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E153" s="3" t="s">
         <v>29</v>
@@ -15519,7 +15521,7 @@
         <v>27</v>
       </c>
       <c r="D154" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E154" s="3" t="s">
         <v>29</v>
@@ -15592,7 +15594,7 @@
         <v>27</v>
       </c>
       <c r="D155" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E155" s="3" t="s">
         <v>29</v>
@@ -15665,7 +15667,7 @@
         <v>27</v>
       </c>
       <c r="D156" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E156" s="3" t="s">
         <v>29</v>
@@ -15815,7 +15817,7 @@
         <v>27</v>
       </c>
       <c r="D158" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E158" s="3" t="s">
         <v>151</v>
@@ -15859,7 +15861,7 @@
       </c>
       <c r="S158" s="3"/>
       <c r="T158" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="U158" s="3" t="s">
         <v>37</v>
@@ -15888,7 +15890,7 @@
         <v>27</v>
       </c>
       <c r="D159" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E159" s="3" t="s">
         <v>151</v>
@@ -15932,7 +15934,7 @@
       </c>
       <c r="S159" s="3"/>
       <c r="T159" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="U159" s="3" t="s">
         <v>37</v>
@@ -15961,7 +15963,7 @@
         <v>27</v>
       </c>
       <c r="D160" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E160" s="3" t="s">
         <v>151</v>
@@ -16034,7 +16036,7 @@
         <v>27</v>
       </c>
       <c r="D161" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E161" s="3" t="s">
         <v>704</v>
@@ -16107,7 +16109,7 @@
         <v>27</v>
       </c>
       <c r="D162" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E162" s="3" t="s">
         <v>704</v>
@@ -16180,7 +16182,7 @@
         <v>27</v>
       </c>
       <c r="D163" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E163" s="3" t="s">
         <v>704</v>
@@ -16253,7 +16255,7 @@
         <v>27</v>
       </c>
       <c r="D164" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E164" s="3" t="s">
         <v>704</v>
@@ -16326,7 +16328,7 @@
         <v>27</v>
       </c>
       <c r="D165" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E165" s="3" t="s">
         <v>704</v>
@@ -16399,7 +16401,7 @@
         <v>27</v>
       </c>
       <c r="D166" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E166" s="3" t="s">
         <v>704</v>
@@ -16472,7 +16474,7 @@
         <v>27</v>
       </c>
       <c r="D167" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E167" s="3" t="s">
         <v>704</v>
@@ -16545,7 +16547,7 @@
         <v>27</v>
       </c>
       <c r="D168" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E168" s="3" t="s">
         <v>704</v>
@@ -16618,7 +16620,7 @@
         <v>27</v>
       </c>
       <c r="D169" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E169" s="3" t="s">
         <v>704</v>
@@ -16691,7 +16693,7 @@
         <v>27</v>
       </c>
       <c r="D170" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E170" s="3" t="s">
         <v>704</v>
@@ -16764,7 +16766,7 @@
         <v>27</v>
       </c>
       <c r="D171" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E171" s="3" t="s">
         <v>704</v>
@@ -16837,7 +16839,7 @@
         <v>27</v>
       </c>
       <c r="D172" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E172" s="3" t="s">
         <v>704</v>
@@ -16910,7 +16912,7 @@
         <v>27</v>
       </c>
       <c r="D173" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E173" s="3" t="s">
         <v>704</v>
@@ -16983,7 +16985,7 @@
         <v>27</v>
       </c>
       <c r="D174" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E174" s="3" t="s">
         <v>704</v>
@@ -17056,7 +17058,7 @@
         <v>27</v>
       </c>
       <c r="D175" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E175" s="3" t="s">
         <v>704</v>
@@ -17129,7 +17131,7 @@
         <v>27</v>
       </c>
       <c r="D176" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E176" s="3" t="s">
         <v>704</v>
@@ -17202,7 +17204,7 @@
         <v>27</v>
       </c>
       <c r="D177" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E177" s="3" t="s">
         <v>704</v>
@@ -17275,7 +17277,7 @@
         <v>27</v>
       </c>
       <c r="D178" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E178" s="3" t="s">
         <v>704</v>
@@ -17348,7 +17350,7 @@
         <v>27</v>
       </c>
       <c r="D179" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E179" s="3" t="s">
         <v>704</v>
@@ -17421,7 +17423,7 @@
         <v>27</v>
       </c>
       <c r="D180" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E180" s="3" t="s">
         <v>704</v>
@@ -17494,7 +17496,7 @@
         <v>27</v>
       </c>
       <c r="D181" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E181" s="3" t="s">
         <v>704</v>
@@ -17567,7 +17569,7 @@
         <v>27</v>
       </c>
       <c r="D182" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E182" s="3" t="s">
         <v>704</v>
@@ -17640,7 +17642,7 @@
         <v>27</v>
       </c>
       <c r="D183" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E183" s="3" t="s">
         <v>704</v>
@@ -17713,7 +17715,7 @@
         <v>27</v>
       </c>
       <c r="D184" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E184" s="3" t="s">
         <v>704</v>
@@ -17786,7 +17788,7 @@
         <v>27</v>
       </c>
       <c r="D185" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E185" s="3" t="s">
         <v>704</v>
@@ -17859,7 +17861,7 @@
         <v>27</v>
       </c>
       <c r="D186" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E186" s="3" t="s">
         <v>704</v>
@@ -17932,7 +17934,7 @@
         <v>27</v>
       </c>
       <c r="D187" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E187" s="3" t="s">
         <v>704</v>
@@ -18005,7 +18007,7 @@
         <v>27</v>
       </c>
       <c r="D188" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E188" s="3" t="s">
         <v>704</v>
@@ -18078,7 +18080,7 @@
         <v>27</v>
       </c>
       <c r="D189" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E189" s="3" t="s">
         <v>704</v>
@@ -18151,7 +18153,7 @@
         <v>27</v>
       </c>
       <c r="D190" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E190" s="3" t="s">
         <v>704</v>
@@ -18224,7 +18226,7 @@
         <v>27</v>
       </c>
       <c r="D191" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E191" s="3" t="s">
         <v>704</v>
@@ -18297,7 +18299,7 @@
         <v>27</v>
       </c>
       <c r="D192" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E192" s="3" t="s">
         <v>704</v>
@@ -18370,7 +18372,7 @@
         <v>27</v>
       </c>
       <c r="D193" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E193" s="3" t="s">
         <v>704</v>
@@ -18443,7 +18445,7 @@
         <v>27</v>
       </c>
       <c r="D194" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E194" s="3" t="s">
         <v>704</v>
@@ -18516,7 +18518,7 @@
         <v>27</v>
       </c>
       <c r="D195" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E195" s="3" t="s">
         <v>704</v>
@@ -18589,7 +18591,7 @@
         <v>27</v>
       </c>
       <c r="D196" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E196" s="3" t="s">
         <v>704</v>
@@ -18662,7 +18664,7 @@
         <v>27</v>
       </c>
       <c r="D197" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E197" s="3" t="s">
         <v>704</v>
@@ -18735,7 +18737,7 @@
         <v>27</v>
       </c>
       <c r="D198" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E198" s="3" t="s">
         <v>704</v>
@@ -18808,7 +18810,7 @@
         <v>27</v>
       </c>
       <c r="D199" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E199" s="3" t="s">
         <v>704</v>
@@ -18881,7 +18883,7 @@
         <v>27</v>
       </c>
       <c r="D200" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E200" s="3" t="s">
         <v>704</v>
@@ -18954,7 +18956,7 @@
         <v>27</v>
       </c>
       <c r="D201" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E201" s="3" t="s">
         <v>704</v>
@@ -18998,7 +19000,7 @@
       </c>
       <c r="S201" s="3"/>
       <c r="T201" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="U201" s="3" t="s">
         <v>37</v>
@@ -19250,7 +19252,7 @@
         <v>27</v>
       </c>
       <c r="D205" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E205" s="3" t="s">
         <v>29</v>
@@ -19294,7 +19296,7 @@
       </c>
       <c r="S205" s="3"/>
       <c r="T205" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="U205" s="3" t="s">
         <v>37</v>
@@ -19396,7 +19398,7 @@
         <v>27</v>
       </c>
       <c r="D207" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E207" s="3" t="s">
         <v>29</v>
@@ -19440,7 +19442,7 @@
       </c>
       <c r="S207" s="3"/>
       <c r="T207" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="U207" s="3" t="s">
         <v>37</v>
@@ -19469,7 +19471,7 @@
         <v>27</v>
       </c>
       <c r="D208" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E208" s="3" t="s">
         <v>29</v>
@@ -19542,7 +19544,7 @@
         <v>27</v>
       </c>
       <c r="D209" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E209" s="3" t="s">
         <v>29</v>
@@ -19615,7 +19617,7 @@
         <v>27</v>
       </c>
       <c r="D210" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E210" s="3" t="s">
         <v>29</v>
@@ -19659,7 +19661,7 @@
       </c>
       <c r="S210" s="3"/>
       <c r="T210" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="U210" s="3" t="s">
         <v>37</v>
@@ -19688,7 +19690,7 @@
         <v>27</v>
       </c>
       <c r="D211" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E211" s="3" t="s">
         <v>29</v>
@@ -20061,7 +20063,7 @@
         <v>27</v>
       </c>
       <c r="D216" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E216" s="3" t="s">
         <v>29</v>
@@ -20132,7 +20134,7 @@
         <v>27</v>
       </c>
       <c r="D217" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E217" s="3" t="s">
         <v>29</v>
@@ -20251,7 +20253,7 @@
         <v>121</v>
       </c>
       <c r="T218" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="U218" s="3" t="s">
         <v>37</v>
@@ -20328,7 +20330,7 @@
         <v>121</v>
       </c>
       <c r="T219" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="U219" s="3" t="s">
         <v>37</v>
@@ -20357,7 +20359,7 @@
         <v>27</v>
       </c>
       <c r="D220" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E220" s="3" t="s">
         <v>29</v>
@@ -20430,7 +20432,7 @@
         <v>27</v>
       </c>
       <c r="D221" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E221" s="3" t="s">
         <v>29</v>
@@ -20801,7 +20803,7 @@
         <v>27</v>
       </c>
       <c r="D226" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E226" s="3" t="s">
         <v>29</v>
@@ -20876,7 +20878,7 @@
         <v>27</v>
       </c>
       <c r="D227" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E227" s="3" t="s">
         <v>29</v>
@@ -20951,7 +20953,7 @@
         <v>27</v>
       </c>
       <c r="D228" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E228" s="3" t="s">
         <v>1120</v>
@@ -21024,7 +21026,7 @@
         <v>27</v>
       </c>
       <c r="D229" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E229" s="3" t="s">
         <v>1120</v>
@@ -21097,7 +21099,7 @@
         <v>27</v>
       </c>
       <c r="D230" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E230" s="3" t="s">
         <v>616</v>
@@ -21170,7 +21172,7 @@
         <v>27</v>
       </c>
       <c r="D231" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E231" s="3" t="s">
         <v>616</v>
@@ -21243,7 +21245,7 @@
         <v>27</v>
       </c>
       <c r="D232" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E232" s="3" t="s">
         <v>29</v>
@@ -21320,7 +21322,7 @@
         <v>27</v>
       </c>
       <c r="D233" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E233" s="3" t="s">
         <v>29</v>
@@ -21397,7 +21399,7 @@
         <v>27</v>
       </c>
       <c r="D234" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E234" s="3" t="s">
         <v>1071</v>
@@ -21470,7 +21472,7 @@
         <v>27</v>
       </c>
       <c r="D235" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E235" s="3" t="s">
         <v>1071</v>
@@ -21543,7 +21545,7 @@
         <v>27</v>
       </c>
       <c r="D236" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E236" s="3" t="s">
         <v>1071</v>
@@ -21616,7 +21618,7 @@
         <v>27</v>
       </c>
       <c r="D237" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E237" s="3" t="s">
         <v>29</v>
@@ -21985,7 +21987,7 @@
         <v>27</v>
       </c>
       <c r="D242" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E242" s="3" t="s">
         <v>1071</v>
@@ -22033,7 +22035,7 @@
         <v>121</v>
       </c>
       <c r="T242" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="U242" s="3" t="s">
         <v>37</v>
@@ -22281,7 +22283,7 @@
         <v>27</v>
       </c>
       <c r="D246" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E246" s="3" t="s">
         <v>29</v>
@@ -22358,7 +22360,7 @@
         <v>27</v>
       </c>
       <c r="D247" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E247" s="3" t="s">
         <v>29</v>
@@ -22581,7 +22583,7 @@
         <v>27</v>
       </c>
       <c r="D250" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E250" s="3" t="s">
         <v>29</v>
@@ -22658,7 +22660,7 @@
         <v>27</v>
       </c>
       <c r="D251" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E251" s="3" t="s">
         <v>29</v>
@@ -22735,7 +22737,7 @@
         <v>27</v>
       </c>
       <c r="D252" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E252" s="3" t="s">
         <v>29</v>
@@ -22810,7 +22812,7 @@
         <v>27</v>
       </c>
       <c r="D253" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E253" s="3" t="s">
         <v>29</v>
@@ -22887,7 +22889,7 @@
         <v>27</v>
       </c>
       <c r="D254" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E254" s="3" t="s">
         <v>1269</v>
@@ -22964,7 +22966,7 @@
         <v>27</v>
       </c>
       <c r="D255" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E255" s="3" t="s">
         <v>1269</v>
@@ -23335,8 +23337,8 @@
       <c r="L3" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="M3" s="6" t="b">
-        <v>0</v>
+      <c r="M3" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="N3" s="5" t="b">
         <v>1</v>
@@ -23356,7 +23358,7 @@
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B4" s="5" t="b">
         <v>1</v>
@@ -23412,7 +23414,7 @@
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B5" s="5" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
generated all the reports on 2026-05-17
</commit_message>
<xml_diff>
--- a/report/merged_configurations.xlsx
+++ b/report/merged_configurations.xlsx
@@ -3899,7 +3899,7 @@
     <t>NDNN-description.md</t>
   </si>
   <si>
-    <t>[{"name":"Implementatiemodel Nudging Down Night Noise","resourceReference":"https://data.vlaanderen.be/doc/implementatiemodel/nudgingdownnightnoise/"}]</t>
+    <t>[{"name":"Implementatiemodel Nudging Down Night Noise","resourceReference":"https://data.vlaanderen.be/doc/implementatiemodel/nudgingdownnightnoise/2026-04-14"}]</t>
   </si>
   <si>
     <t>Charter NDNN</t>
@@ -24763,7 +24763,7 @@
         <v>31</v>
       </c>
       <c r="F258" s="4">
-        <v>46129</v>
+        <v>46126</v>
       </c>
       <c r="G258" s="3" t="s">
         <v>1294</v>

</xml_diff>

<commit_message>
generated all the reports on 2026-05-24
</commit_message>
<xml_diff>
--- a/report/merged_configurations.xlsx
+++ b/report/merged_configurations.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5843" uniqueCount="1302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5843" uniqueCount="1301">
   <si>
     <t>title</t>
   </si>
@@ -3899,7 +3899,7 @@
     <t>NDNN-description.md</t>
   </si>
   <si>
-    <t>[{"name":"Implementatiemodel Nudging Down Night Noise","resourceReference":"https://data.vlaanderen.be/doc/implementatiemodel/nudgingdownnightnoise/2026-04-14"}]</t>
+    <t>[{"name":"Implementatiemodel Nudging Down Night Noise","resourceReference":"https://data.vlaanderen.be/doc/implementatiemodel/geluidsmeldingen-en-geluidsmetingen/ontwerpstandaard/2026-05-20"}]</t>
   </si>
   <si>
     <t>Charter NDNN</t>
@@ -3912,9 +3912,6 @@
   </si>
   <si>
     <t>[{"name":"Presentatie Business Werkgroep -  5 maart 2026","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-NDNN/standaardenregister/presentations/Presentatie%20Business%20Werkgroep%20NDNN%2005-03-2026.pdf"},{"name":"Presentatie Thematische Werkgroep - 2 April 2026","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-NDNN/standaardenregister/presentations/Presentatie%20Thematische%20werkgroep%201%20NDNN%2002-04-2026.pdf"}]</t>
-  </si>
-  <si>
-    <t>https://data.vlaanderen.be/id/concept/Domein/Werk</t>
   </si>
   <si>
     <t>{"name":"Charter NDNN","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-NDNN/standaardenregister/charter/Werkgroep%20charter%20OSLO_NudgingDownNightNoise.pdf"}</t>
@@ -8257,7 +8254,7 @@
         <v>310</v>
       </c>
       <c r="F50" s="4">
-        <v>44679</v>
+        <v>45546</v>
       </c>
       <c r="G50" s="3" t="s">
         <v>311</v>
@@ -8324,7 +8321,7 @@
         <v>322</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>28</v>
+        <v>76</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>29</v>
@@ -8336,7 +8333,7 @@
         <v>310</v>
       </c>
       <c r="F51" s="4">
-        <v>44679</v>
+        <v>45546</v>
       </c>
       <c r="G51" s="3" t="s">
         <v>323</v>
@@ -24795,7 +24792,7 @@
       <c r="R258" s="3"/>
       <c r="S258" s="3"/>
       <c r="T258" s="3" t="s">
-        <v>1300</v>
+        <v>90</v>
       </c>
       <c r="U258" s="3" t="s">
         <v>34</v>
@@ -24807,7 +24804,7 @@
         <v>39</v>
       </c>
       <c r="X258" s="3" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
       <c r="Y258" s="3" t="s">
         <v>39</v>

</xml_diff>

<commit_message>
generated all the reports on 2026-06-07
</commit_message>
<xml_diff>
--- a/report/merged_configurations.xlsx
+++ b/report/merged_configurations.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5843" uniqueCount="1301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5843" uniqueCount="1303">
   <si>
     <t>title</t>
   </si>
@@ -3863,7 +3863,7 @@
     <t>Vocabularium Rooilijnplannen</t>
   </si>
   <si>
-    <t>OSLO SSN SOSA VL</t>
+    <t>SSN SOSA VL</t>
   </si>
   <si>
     <t>https://data.vlaanderen.be/id/concept/StandaardType/Interoperabiliteit</t>
@@ -3915,6 +3915,12 @@
   </si>
   <si>
     <t>{"name":"Charter NDNN","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-NDNN/standaardenregister/charter/Werkgroep%20charter%20OSLO_NudgingDownNightNoise.pdf"}</t>
+  </si>
+  <si>
+    <t>[{"name":"OSLO SSN SOSA","resourceReference":"https://data.vlaanderen.be/standaarden/oslo-ssn-sosa-vl"},{"name":"OSLO Melding","resourceReference":"https://data.vlaanderen.be/ns/melding/"},{"name":"OSLO Verkeersmeldingen","resourceReference":"https://data.vlaanderen.be/doc/implementatiemodel/verkeersmeldingen/"},{"name":"OSLO Omgevingsvergunning","resourceReference":"https://data.vlaanderen.be/doc/applicatieprofiel/omgevingsvergunning/"},{"name":"OSLO Dossier","resourceReference":"https://data.vlaanderen.be/doc/applicatieprofiel/dossier/"},{"name":"OSLO Generiek","resourceReference":"https://data.vlaanderen.be/doc/applicatieprofiel/generiek-basis/"}]</t>
+  </si>
+  <si>
+    <t>[{"name":"Overzicht use cases","resourceReference":"https://github.com/Informatievlaanderen/OSLOthema-NDNN/blob/main/usecases.md"}]</t>
   </si>
 </sst>
 </file>
@@ -16792,7 +16798,7 @@
         <v>153</v>
       </c>
       <c r="F158" s="4">
-        <v>46073</v>
+        <v>46065</v>
       </c>
       <c r="G158" s="3" t="s">
         <v>823</v>
@@ -16822,7 +16828,7 @@
         <v>46030</v>
       </c>
       <c r="P158" s="4">
-        <v>46073</v>
+        <v>46065</v>
       </c>
       <c r="Q158" s="3"/>
       <c r="R158" s="3" t="s">
@@ -16871,7 +16877,7 @@
         <v>153</v>
       </c>
       <c r="F159" s="4">
-        <v>46073</v>
+        <v>46065</v>
       </c>
       <c r="G159" s="3" t="s">
         <v>823</v>
@@ -16901,7 +16907,7 @@
         <v>46030</v>
       </c>
       <c r="P159" s="4">
-        <v>46073</v>
+        <v>46065</v>
       </c>
       <c r="Q159" s="3"/>
       <c r="R159" s="3" t="s">
@@ -24810,10 +24816,10 @@
         <v>39</v>
       </c>
       <c r="Z258" s="3" t="s">
-        <v>34</v>
+        <v>1301</v>
       </c>
       <c r="AA258" s="3" t="s">
-        <v>34</v>
+        <v>1302</v>
       </c>
     </row>
   </sheetData>

</xml_diff>